<commit_message>
Feature: pantalla Objetivo alimentada por el Sheet + simulador de interés compuesto
La cartera, nombre, fecha límite y monto del objetivo ahora se cargan en una
pestaña nueva del Sheet ("Objetivos") en vez de un modal en la app, siguiendo
el mismo patrón espejo que Movimientos/Instrumentos/Precios. Se agrega además
un simulador de tasa de interés anual (100% cliente) que recalcula el aporte
mensual necesario y cuántos meses/aportes se ahorran con ese interés.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheet_local/sheet_inversiones.xlsx
+++ b/sheet_local/sheet_inversiones.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Movimientos" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Instrumentos" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Precios" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Objetivos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,9 +19,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -51,9 +51,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -490,7 +491,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -528,12 +529,9 @@
       <c r="J2" t="n">
         <v>1521.33</v>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -571,12 +569,9 @@
       <c r="J3" t="n">
         <v>1521.33</v>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>46205</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -614,12 +609,9 @@
       <c r="J4" t="n">
         <v>1529.77</v>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>46205</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -657,12 +649,9 @@
       <c r="J5" t="n">
         <v>1529.77</v>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>46205</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -700,12 +689,9 @@
       <c r="J6" t="n">
         <v>1529.77</v>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>46205</v>
       </c>
       <c r="B7" t="inlineStr">
@@ -743,12 +729,9 @@
       <c r="J7" t="n">
         <v>1529.77</v>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="B8" t="inlineStr">
@@ -786,12 +769,9 @@
       <c r="J8" t="n">
         <v>1524.53</v>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="B9" t="inlineStr">
@@ -829,14 +809,12 @@
       <c r="J9" t="n">
         <v>1516.89</v>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
         <v>90845</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="B10" t="inlineStr">
@@ -874,14 +852,12 @@
       <c r="J10" t="n">
         <v>1516.89</v>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
         <v>59.80579329</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="B11" t="inlineStr">
@@ -919,12 +895,9 @@
       <c r="J11" t="n">
         <v>1516.89</v>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="B12" t="inlineStr">
@@ -962,12 +935,9 @@
       <c r="J12" t="n">
         <v>1516.89</v>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="B13" t="inlineStr">
@@ -1005,9 +975,6 @@
       <c r="J13" t="n">
         <v>1516.89</v>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1121,7 +1088,6 @@
           <t>Energía</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>Porcentaje</t>
@@ -1130,8 +1096,6 @@
       <c r="J2" t="n">
         <v>20</v>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1169,11 +1133,6 @@
           <t>Soberano</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1211,11 +1170,6 @@
           <t>Soberano</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1253,11 +1207,6 @@
           <t>Liquidez</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1295,11 +1244,6 @@
           <t>Indice</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1337,9 +1281,6 @@
           <t>Cosumo Masivo</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>Fijo</t>
@@ -1385,7 +1326,6 @@
           <t>Tecnologia</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>Porcentaje</t>
@@ -1460,7 +1400,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>46227</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -1482,13 +1422,12 @@
       <c r="F2" t="n">
         <v>1530.38</v>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
         <v>95240</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>46227</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -1510,13 +1449,12 @@
       <c r="F3" t="n">
         <v>1530.38</v>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
         <v>62.23290947</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>46227</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -1538,11 +1476,9 @@
       <c r="F4" t="n">
         <v>1530.38</v>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>46227</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -1564,11 +1500,9 @@
       <c r="F5" t="n">
         <v>1530.38</v>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>46230</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -1590,13 +1524,12 @@
       <c r="F6" t="n">
         <v>1532.78</v>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
         <v>0.04058313713</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>46230</v>
       </c>
       <c r="B7" t="inlineStr">
@@ -1618,11 +1551,9 @@
       <c r="F7" t="n">
         <v>1532.78</v>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>46230</v>
       </c>
       <c r="B8" t="inlineStr">
@@ -1644,11 +1575,9 @@
       <c r="F8" t="n">
         <v>1532.78</v>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>46230</v>
       </c>
       <c r="B9" t="inlineStr">
@@ -1670,11 +1599,9 @@
       <c r="F9" t="n">
         <v>1532.78</v>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="B10" t="inlineStr">
@@ -1696,11 +1623,9 @@
       <c r="F10" t="n">
         <v>1516.89</v>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="B11" t="inlineStr">
@@ -1722,11 +1647,9 @@
       <c r="F11" t="n">
         <v>1516.89</v>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="B12" t="inlineStr">
@@ -1748,11 +1671,9 @@
       <c r="F12" t="n">
         <v>1516.89</v>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="B13" t="inlineStr">
@@ -1774,11 +1695,9 @@
       <c r="F13" t="n">
         <v>1516.89</v>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="B14" t="inlineStr">
@@ -1800,11 +1719,9 @@
       <c r="F14" t="n">
         <v>1516.89</v>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="B15" t="inlineStr">
@@ -1826,8 +1743,122 @@
       <c r="F15" t="n">
         <v>1516.89</v>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Cartera</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Fecha Límite</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Monto USD</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Icono</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Fondo de emergencia</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Fondo de emergencia</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>🚨</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Jubilación (30 años)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Jubilación</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2056-01-01</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>🏖️</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Preservación de Capital</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2028-06-01</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>40000</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>🏠</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Feature: pantalla Balance de Cartera con objetivos de rebalanceo
Nueva pestaña Rebalanceo en el Sheet para fijar % objetivo de asignación
en 3 ejes independientes (Cartera, Tipo, Sector) y pantalla nueva que
compara el % actual contra el objetivo, con las categorías sin objetivo
agrupadas aparte. De paso corrige el % del eje Sector en Exposición, que
se calculaba sobre el subtotal con sector cargado en vez del total real
de la cartera.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheet_local/sheet_inversiones.xlsx
+++ b/sheet_local/sheet_inversiones.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Instrumentos" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Precios" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Objetivos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Rebalanceo" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1863,4 +1864,260 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Cartera</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Eje</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Categoría</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Porcentaje Objetivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Consolidado</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Cartera</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Fondo de emergencia</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Consolidado</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Cartera</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Jubilación (30 años)</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Consolidado</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cartera</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Preservación de Capital</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Fondo de emergencia</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>FCI</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Preservación de Capital</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Bono</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Preservación de Capital</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CEDEAR</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Jubilación (30 años)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CEDEAR</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Jubilación (30 años)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Tecnologia</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Jubilación (30 años)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Cosumo Masivo</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Jubilación (30 años)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Indice</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Jubilación (30 años)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Energía</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Feature: motor de métricas de riesgo (drawdown, volatilidad, Sharpe, Sortino, Calmar)
Agrega un motor puro de riesgo (risk_engine.py) sobre el TWR mensual encadenado
existente, con estado explícito de "datos insuficientes" por métrica. Sharpe se
calcula contra un benchmark elegido por el usuario, alimentado por una nueva
pestaña Benchmarks en el Sheet (Fecha | Benchmark | Valor). Nueva pantalla
Riesgo (drawdown underwater, volatilidad, Sharpe/Sortino/Calmar, mejores/peores
meses), enlazada desde Rendimiento. Bootstrapea pytest con 17 tests numéricos.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheet_local/sheet_inversiones.xlsx
+++ b/sheet_local/sheet_inversiones.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Precios" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Objetivos" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Rebalanceo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Benchmarks" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2120,4 +2121,86 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Benchmark</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2024-01-31</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MERVAL</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2024-02-29</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MERVAL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2024-03-31</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MERVAL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix: Benchmark configuration and MEP/CER data loading
- Fix NaN handling in Excel reader to avoid 'nan' strings in database
- Add Configuracion tab with benchmarks for each cartera (MERVAL)
- Add NULL cartera row for consolidado benchmark
- Add historical MEP/CER data for FX decomposition
- Aggregate objectives from Google Sheets when available

Changes:
- sheets_client.py: Convert NaN to empty string instead of 'nan'
- sheet_inversiones.xlsx: Added Configuracion tab with benchmark setup

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheet_local/sheet_inversiones.xlsx
+++ b/sheet_local/sheet_inversiones.xlsx
@@ -8,11 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Movimientos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Instrumentos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Precios" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Objetivos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rebalanceo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Benchmarks" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Tipos de Cambio" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Instrumentos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Precios" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Objetivos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Rebalanceo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Benchmarks" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Configuracion" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +26,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,13 +34,22 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D3D3D3"/>
+        <bgColor rgb="00D3D3D3"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -53,10 +64,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -989,360 +1001,209 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Nombre</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Tipo Instrumento</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Mercado</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Moneda</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>País</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Sector</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Fecha Vencimiento</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Objetivo Modo</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Objetivo Valor</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Stop Loss Modo</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Stop Loss Valor</t>
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Valor</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Energy Sector ETF</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CEDEAR</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>AR</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Energía</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Porcentaje</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>20</v>
+          <t>MEP</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>818</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TZXD7</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Boncer 2027 (CER +0%)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Bono</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>MERVAL</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>AR</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Soberano</t>
-        </is>
+          <t>CER</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>103.6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>S30S6</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Setea Sep 2026 (2.53%)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Bono</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>MERVAL</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>AR</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Soberano</t>
-        </is>
+          <t>MEP</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>815</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1810 Ahorros Activos</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>FCI Money Market</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>FCI</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>MERVAL</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>AR</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Liquidez</t>
-        </is>
+          <t>CER</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>103</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SYP</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Indice</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CEDEAR</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>AR</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Indice</t>
-        </is>
+          <t>MEP</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>812</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Consumo Masivo</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CEDEAR</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>AR</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Cosumo Masivo</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="L7" t="n">
-        <v>25000</v>
+          <t>CER</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>102.4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tecnologia</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CEDEAR</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>AR</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Tecnologia</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Porcentaje</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>15</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Porcentaje</t>
-        </is>
-      </c>
-      <c r="L8" t="n">
-        <v>-10</v>
+          <t>MEP</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CER</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>101.8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MEP</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CER</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>101.2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>MEP</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CER</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>100.6</v>
       </c>
     </row>
   </sheetData>
@@ -1356,394 +1217,360 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Fecha</t>
+          <t>Ticker</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Ticker</t>
+          <t>Nombre</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Precio</t>
+          <t>Tipo Instrumento</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Mercado</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Moneda</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>CER</t>
-        </is>
-      </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>MEP</t>
+          <t>País</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Unnamed: 6</t>
+          <t>Sector</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Unnamed: 7</t>
+          <t>Fecha Vencimiento</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Objetivo Modo</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Objetivo Valor</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Stop Loss Modo</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Stop Loss Valor</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>46227</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>XLE</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>XLE</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>47620</v>
+          <t>Energy Sector ETF</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CEDEAR</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>811.9761999999999</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1530.38</v>
-      </c>
-      <c r="H2" t="n">
-        <v>95240</v>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Energía</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Porcentaje</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>46227</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TZXD7</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TZXD7</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>2.7105</v>
+          <t>Boncer 2027 (CER +0%)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Bono</t>
+        </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>811.9761999999999</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1530.38</v>
-      </c>
-      <c r="H3" t="n">
-        <v>62.23290947</v>
+          <t>MERVAL</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Soberano</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>46227</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S30S6</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>S30S6</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>1.1283</v>
+          <t>Setea Sep 2026 (2.53%)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Bono</t>
+        </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>811.9761999999999</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1530.38</v>
+          <t>MERVAL</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Soberano</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>46227</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1810 Ahorros Activos</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1810 Ahorros Activos</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>30.01</v>
+          <t>FCI Money Market</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>FCI</t>
+        </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>811.9761999999999</v>
-      </c>
-      <c r="F5" t="n">
-        <v>1530.38</v>
+          <t>MERVAL</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Liquidez</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>46230</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SYP</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>XLE</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>46880</v>
+          <t>Indice</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CEDEAR</t>
+        </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>813.4565</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1532.78</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.04058313713</v>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Indice</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>46230</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TZXD7</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>2.7135</v>
+          <t>Consumo Masivo</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CEDEAR</t>
+        </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>813.4565</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1532.78</v>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Cosumo Masivo</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>25000</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>46230</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>S30S6</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>1.12909</v>
+          <t>Tecnologia</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CEDEAR</t>
+        </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>813.4565</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1532.78</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>46230</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>1810 Ahorros Activos</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>30.084208</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>813.4565</v>
-      </c>
-      <c r="F9" t="n">
-        <v>1532.78</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>XLE</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>46600</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>815.4299999999999</v>
-      </c>
-      <c r="F10" t="n">
-        <v>1516.89</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>TZXD7</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>2.71</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>815.4299999999999</v>
-      </c>
-      <c r="F11" t="n">
-        <v>1516.89</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>S30S6</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>1.1305</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>815.4299999999999</v>
-      </c>
-      <c r="F12" t="n">
-        <v>1516.89</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>SYP</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>19620</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>815.4299999999999</v>
-      </c>
-      <c r="F13" t="n">
-        <v>1516.89</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>27440</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>815.4299999999999</v>
-      </c>
-      <c r="F14" t="n">
-        <v>1516.89</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>MSFT</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>24280</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>815.4299999999999</v>
-      </c>
-      <c r="F15" t="n">
-        <v>1516.89</v>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Tecnologia</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Porcentaje</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>15</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Porcentaje</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>-10</v>
       </c>
     </row>
   </sheetData>
@@ -1757,109 +1584,394 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Cartera</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Nombre</t>
+          <t>Ticker</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Fecha Límite</t>
+          <t>Precio</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Monto USD</t>
+          <t>Moneda</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Icono</t>
+          <t>CER</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>MEP</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Unnamed: 6</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Unnamed: 7</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Fondo de emergencia</t>
-        </is>
+      <c r="A2" s="2" t="n">
+        <v>46227</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Fondo de emergencia</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>🚨</t>
-        </is>
+          <t>XLE</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>47620</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>811.9761999999999</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1530.38</v>
+      </c>
+      <c r="H2" t="n">
+        <v>95240</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Jubilación (30 años)</t>
-        </is>
+      <c r="A3" s="2" t="n">
+        <v>46227</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Jubilación</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2056-01-01</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>500000</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>🏖️</t>
-        </is>
+          <t>TZXD7</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2.7105</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>811.9761999999999</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1530.38</v>
+      </c>
+      <c r="H3" t="n">
+        <v>62.23290947</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Preservación de Capital</t>
-        </is>
+      <c r="A4" s="2" t="n">
+        <v>46227</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Casa</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2028-06-01</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>40000</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>🏠</t>
-        </is>
+          <t>S30S6</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1.1283</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>811.9761999999999</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1530.38</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1810 Ahorros Activos</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>30.01</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>811.9761999999999</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1530.38</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>XLE</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>46880</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>813.4565</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1532.78</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.04058313713</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TZXD7</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2.7135</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>813.4565</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1532.78</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>S30S6</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1.12909</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>813.4565</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1532.78</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1810 Ahorros Activos</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>30.084208</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>813.4565</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1532.78</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>XLE</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>46600</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>815.4299999999999</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1516.89</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TZXD7</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>815.4299999999999</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1516.89</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>S30S6</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1.1305</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>815.4299999999999</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1516.89</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>SYP</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>19620</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>815.4299999999999</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1516.89</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>27440</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>815.4299999999999</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1516.89</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>24280</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>815.4299999999999</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1516.89</v>
       </c>
     </row>
   </sheetData>
@@ -1873,7 +1985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1884,238 +1996,98 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Eje</t>
+          <t>Nombre</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Categoría</t>
+          <t>Fecha Límite</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Porcentaje Objetivo</t>
+          <t>Monto USD</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Icono</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Consolidado</t>
+          <t>Fondo de emergencia</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cartera</t>
+          <t>Fondo de emergencia</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fondo de emergencia</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>30</v>
+        <v>5000</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>🚨</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Consolidado</t>
+          <t>Jubilación (30 años)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cartera</t>
+          <t>Jubilación</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Jubilación (30 años)</t>
+          <t>2056-01-01</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>50</v>
+        <v>500000</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>🏖️</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Consolidado</t>
+          <t>Preservación de Capital</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cartera</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Preservación de Capital</t>
+          <t>2028-06-01</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Fondo de emergencia</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Tipo</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>FCI</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Preservación de Capital</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Tipo</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Bono</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Preservación de Capital</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Tipo</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CEDEAR</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Jubilación (30 años)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Tipo</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CEDEAR</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Jubilación (30 años)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Sector</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Tecnologia</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Jubilación (30 años)</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Sector</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Cosumo Masivo</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Jubilación (30 años)</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Sector</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Indice</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Jubilación (30 años)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Sector</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Energía</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>15</v>
+        <v>40000</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>🏠</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2129,6 +2101,262 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Cartera</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Eje</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Categoría</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Porcentaje Objetivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Consolidado</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Cartera</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Fondo de emergencia</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Consolidado</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Cartera</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Jubilación (30 años)</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Consolidado</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cartera</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Preservación de Capital</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Fondo de emergencia</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>FCI</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Preservación de Capital</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Bono</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Preservación de Capital</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CEDEAR</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Jubilación (30 años)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CEDEAR</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Jubilación (30 años)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Tecnologia</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Jubilación (30 años)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Cosumo Masivo</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Jubilación (30 años)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Indice</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Jubilación (30 años)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Energía</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -2203,4 +2431,98 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Cartera</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Benchmark</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Rendimiento Objetivo</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Peso Máximo</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Peso Mínimo</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Tolerancia</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MERVAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Fondo de emergencia</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MERVAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Jubilación (30 años)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MERVAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Preservación de Capital</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MERVAL</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>